<commit_message>
July 27: Updated code to use Anthropic's Claude
</commit_message>
<xml_diff>
--- a/output/papua_microbial_sustainability_matrix.xlsx
+++ b/output/papua_microbial_sustainability_matrix.xlsx
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Methyloceanibacter caenitepidi</t>
+          <t>1 Methyloceanibacter caenitepidi</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -463,7 +463,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Thermomarinilinea lacunifontana</t>
+          <t>2 Thermomarinilinea lacunifontana</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -485,7 +485,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Litorilinea aerophila</t>
+          <t>3 Litorilinea aerophila</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -507,7 +507,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Filomicrobium fusiforme</t>
+          <t>4 Filomicrobium fusiforme</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -529,7 +529,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Desulfofustis glycolicus</t>
+          <t>5 Desulfofustis glycolicus</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -551,7 +551,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Dehalococcoides mccartyi</t>
+          <t>6 Dehalococcoides mccartyi</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -573,7 +573,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Methylothermalis aethiopiae</t>
+          <t>7 Methylothermalis aethiopiae</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -595,7 +595,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Symbiobacterium terraclitae</t>
+          <t>8 Symbiobacterium terraclitae</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Ilumatobacter fluminis</t>
+          <t>9 Ilumatobacter fluminis</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Filomicrobium insigne</t>
+          <t>10 Filomicrobium insigne</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -661,7 +661,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Fischerella indica</t>
+          <t>11 Fischerella indica</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -683,7 +683,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Anaerolinea thermophila</t>
+          <t>12 Anaerolinea thermophila</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -705,7 +705,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Rhodoplanes tepidicaeni</t>
+          <t>13 Rhodoplanes tepidicaeni</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -727,7 +727,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Gaiella occulta</t>
+          <t>14 Gaiella occulta</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -749,7 +749,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Mycolicibacterium confluentis</t>
+          <t>15 Mycolicibacterium confluentis</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -771,7 +771,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Hyphomicrobium chloromethanicum</t>
+          <t>16 Hyphomicrobium chloromethanicum</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -793,7 +793,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Psychroglaciecola arctica</t>
+          <t>17 Psychroglaciecola arctica</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -815,7 +815,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Ornithinimicrobium laminariae</t>
+          <t>18 Ornithinimicrobium laminariae</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -837,7 +837,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Pedomicrobium manganicum</t>
+          <t>19 Pedomicrobium manganicum</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -859,7 +859,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Desulfomonile limimaris</t>
+          <t>20 Desulfomonile limimaris</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -881,7 +881,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Iamia majanohamensis</t>
+          <t>21 Iamia majanohamensis</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -903,7 +903,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ktedonosporobacter rubrisoli</t>
+          <t>22 Ktedonosporobacter rubrisoli</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -925,7 +925,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Hydrogenispora ethanolica</t>
+          <t>23 Hydrogenispora ethanolica</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -947,7 +947,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Hoeflea prorocentri</t>
+          <t>24 Hoeflea prorocentri</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -969,7 +969,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Rhabdothermincola salaria</t>
+          <t>25 Rhabdothermincola salaria</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -991,7 +991,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Romboutsia hominis</t>
+          <t>26 Romboutsia hominis</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1013,7 +1013,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Aquihabitans daechungensis</t>
+          <t>27 Aquihabitans daechungensis</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1035,7 +1035,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Nostocoides japonicum</t>
+          <t>28 Nostocoides japonicum</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1057,7 +1057,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Flexilinea flocculi</t>
+          <t>29 Flexilinea flocculi</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1079,7 +1079,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Corynebacterium xerosis</t>
+          <t>30 Corynebacterium xerosis</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1101,7 +1101,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Candidatus Thiodictyon syntrophicum</t>
+          <t>31 Candidatus Thiodictyon syntrophicum</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1123,7 +1123,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Corynebacterium incognita</t>
+          <t>32 Corynebacterium incognita</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1145,7 +1145,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Andreesenia angusta</t>
+          <t>33 Andreesenia angusta</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1167,7 +1167,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Nigerium massiliense</t>
+          <t>34 Nigerium massiliense</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1189,7 +1189,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Conexibacter arvalis</t>
+          <t>35 Conexibacter arvalis</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1211,7 +1211,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Miltoncostaea oceani</t>
+          <t>36 Miltoncostaea oceani</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1233,7 +1233,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Rhabdothermincola sediminis</t>
+          <t>37 Rhabdothermincola sediminis</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1255,7 +1255,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Pseudolabrys taiwanensis</t>
+          <t>38 Pseudolabrys taiwanensis</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Dichotomicrobium thermohalophilum</t>
+          <t>39 Dichotomicrobium thermohalophilum</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1299,7 +1299,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Streptomyces antibioticus</t>
+          <t>40 Streptomyces antibioticus</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1321,7 +1321,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Roseitalea porphyridii</t>
+          <t>41 Roseitalea porphyridii</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1343,7 +1343,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Lignipirellula cremea</t>
+          <t>42 Lignipirellula cremea</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1365,7 +1365,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Zhenhengia yiwuensis</t>
+          <t>43 Zhenhengia yiwuensis</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1387,7 +1387,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Microbaculum marinum</t>
+          <t>44 Microbaculum marinum</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1409,7 +1409,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Sporobacter termitidis</t>
+          <t>45 Sporobacter termitidis</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1431,7 +1431,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Parasynechococcus marenigrum</t>
+          <t>46 Parasynechococcus marenigrum</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1453,7 +1453,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Simkania negevensis</t>
+          <t>47 Simkania negevensis</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1475,7 +1475,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Hyphomicrobium sulfonivorans</t>
+          <t>48 Hyphomicrobium sulfonivorans</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1497,7 +1497,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Prochlorococcus marinus</t>
+          <t>49 Prochlorococcus marinus</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1519,7 +1519,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Hyphomicrobium album</t>
+          <t>50 Hyphomicrobium album</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1541,7 +1541,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Mycobacterium conspicuum</t>
+          <t>51 Mycobacterium conspicuum</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1563,7 +1563,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Salaquimonas pukyongi</t>
+          <t>52 Salaquimonas pukyongi</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1585,7 +1585,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Clostridium estertheticum</t>
+          <t>53 Clostridium estertheticum</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1607,7 +1607,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Pelolinea submarina</t>
+          <t>54 Pelolinea submarina</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1629,7 +1629,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Afifella pfennigii</t>
+          <t>55 Afifella pfennigii</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1651,7 +1651,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Bauldia consociata</t>
+          <t>56 Bauldia consociata</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1673,7 +1673,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Hyphomicrobium hollandicum</t>
+          <t>57 Hyphomicrobium hollandicum</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1695,7 +1695,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Miltoncostaea marina</t>
+          <t>58 Miltoncostaea marina</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1717,7 +1717,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Mycetocola tolaasinivorans</t>
+          <t>59 Mycetocola tolaasinivorans</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1739,7 +1739,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Waddlia chondrophila</t>
+          <t>60 Waddlia chondrophila</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1761,7 +1761,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Algorimarina butyrica</t>
+          <t>61 Algorimarina butyrica</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1783,7 +1783,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Bellilinea caldifistulae</t>
+          <t>62 Bellilinea caldifistulae</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1805,7 +1805,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Caldilinea tarbellica</t>
+          <t>63 Caldilinea tarbellica</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1827,7 +1827,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Bauldia litoralis</t>
+          <t>64 Bauldia litoralis</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1849,7 +1849,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Phycicoccus endophyticus</t>
+          <t>65 Phycicoccus endophyticus</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1871,7 +1871,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Desulfatitalea tepidiphila</t>
+          <t>66 Desulfatitalea tepidiphila</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -1893,7 +1893,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Thermogutta terrifontis</t>
+          <t>67 Thermogutta terrifontis</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -1915,7 +1915,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Pseudorhodoplanes sinuspersici</t>
+          <t>68 Pseudorhodoplanes sinuspersici</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -1937,7 +1937,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Oceanirhabdus sediminicola</t>
+          <t>69 Oceanirhabdus sediminicola</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -1959,7 +1959,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Thiorhodococcus minor</t>
+          <t>70 Thiorhodococcus minor</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -1981,7 +1981,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Desulfomonile tiedjei</t>
+          <t>71 Desulfomonile tiedjei</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2003,7 +2003,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Waddlia malaysiensis</t>
+          <t>72 Waddlia malaysiensis</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2025,7 +2025,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Konateibacter massiliensis</t>
+          <t>73 Konateibacter massiliensis</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2047,7 +2047,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Pirellulimonas nuda</t>
+          <t>74 Pirellulimonas nuda</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2069,7 +2069,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Rhodoplanes pokkaliisoli</t>
+          <t>75 Rhodoplanes pokkaliisoli</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2091,7 +2091,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Rosistilla oblonga</t>
+          <t>76 Rosistilla oblonga</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2113,7 +2113,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Woeseia oceani</t>
+          <t>77 Woeseia oceani</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2135,7 +2135,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Vampirovibrio chlorellavorus</t>
+          <t>78 Vampirovibrio chlorellavorus</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2157,7 +2157,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Clostridium perfringens</t>
+          <t>79 Clostridium perfringens</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2179,7 +2179,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Staphylococcus gallinarum</t>
+          <t>80 Staphylococcus gallinarum</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2201,7 +2201,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Raineyella fluvialis</t>
+          <t>81 Raineyella fluvialis</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2223,7 +2223,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Symmachiella dynata</t>
+          <t>82 Symmachiella dynata</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2245,7 +2245,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Aliiruegeria lutimaris</t>
+          <t>83 Aliiruegeria lutimaris</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Thermanaerothrix daxensis</t>
+          <t>84 Thermanaerothrix daxensis</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2289,7 +2289,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Actinoplanes siamensis</t>
+          <t>85 Actinoplanes siamensis</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2311,7 +2311,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Thiohalocapsa halophila</t>
+          <t>86 Thiohalocapsa halophila</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2333,7 +2333,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Symbioplanes lichenis</t>
+          <t>87 Symbioplanes lichenis</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2355,7 +2355,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Aureliella helgolandensis</t>
+          <t>88 Aureliella helgolandensis</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2377,7 +2377,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Hansschlegelia zhihuaiae</t>
+          <t>89 Hansschlegelia zhihuaiae</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2399,7 +2399,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Romboutsia lituseburensis</t>
+          <t>90 Romboutsia lituseburensis</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2421,7 +2421,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Posidoniimonas corsicana</t>
+          <t>91 Posidoniimonas corsicana</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2443,7 +2443,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Clostridium chrysemydis</t>
+          <t>92 Clostridium chrysemydis</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2465,7 +2465,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Microbacterium halophilum</t>
+          <t>93 Microbacterium halophilum</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2487,7 +2487,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Thiococcus pfennigii</t>
+          <t>94 Thiococcus pfennigii</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2509,7 +2509,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Solirubrobacter soli</t>
+          <t>95 Solirubrobacter soli</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2531,7 +2531,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Mycolicibacterium gadium</t>
+          <t>96 Mycolicibacterium gadium</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2553,7 +2553,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Oricola indica</t>
+          <t>97 Oricola indica</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2575,7 +2575,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Clostridium paraputrificum</t>
+          <t>98 Clostridium paraputrificum</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2597,7 +2597,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Candidatus Protochlamydia naegleriophila</t>
+          <t>99 Candidatus Protochlamydia naegleriophila</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2619,7 +2619,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Jatrophihabitans telluris</t>
+          <t>100 Jatrophihabitans telluris</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">

</xml_diff>

<commit_message>
August 15: Command-Line Interface (CLI) Integration
</commit_message>
<xml_diff>
--- a/output/papua_microbial_sustainability_matrix.xlsx
+++ b/output/papua_microbial_sustainability_matrix.xlsx
@@ -441,677 +441,677 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1 Methyloceanibacter caenitepidi</t>
+          <t>Methyloceanibacter caenitepidi</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Methane oxidation, contributing to the global carbon cycle by converting methane into carbon dioxide</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bioremediation of methane emissions, production of biofuels, and development of eco-friendly technologies for greenhouse gas mitigation</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2 Thermomarinilinea lacunifontana</t>
+          <t>Thermomarinilinea lacunifontana</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Thermomarinilinea lacunifontana is a thermophilic, filamentous bacterium that plays a role in the degradation of organic matter and production of bioactive compounds</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>It has potential applications in sustainable biotechnology, such as bioremediation of polluted environments, production of biofuels, and development of novel therapeutics</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>3 Litorilinea aerophila</t>
+          <t>Litorilinea aerophila</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Aerobic, filamentous bacterium involved in organic matter decomposition and carbon cycling in aquatic environments</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Potential applications in bioremediation of polluted water, production of bioactive compounds, and development of sustainable aquaculture practices</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>4 Filomicrobium fusiforme</t>
+          <t>Filomicrobium fusiforme</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Nitrogen fixation, plant growth promotion, and degradation of organic pollutants</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Biofertilizers, bioremediation of contaminated soil and water, and development of sustainable agricultural practices</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>5 Desulfofustis glycolicus</t>
+          <t>Desulfofustis glycolicus</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Sulfate-reducing bacterium that plays a role in the degradation of organic matter and the sulfur cycle</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bioremediation of contaminated soil and groundwater, production of biofuels and bioproducts, and potential use in sustainable agriculture practices</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>6 Dehalococcoides mccartyi</t>
+          <t>Dehalococcoides mccartyi</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Chlorinated organic compound degradation and reductive dehalogenation</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bioremediation of contaminated soil and groundwater, potential for use in eco-friendly technologies for toxic waste cleanup</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-2</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>7 Methylothermalis aethiopiae</t>
+          <t>Methylothermalis aethiopiae</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Methane oxidation and methanogenesis, contributing to the global carbon cycle</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bioremediation of methane emissions, production of biofuels, and development of sustainable agriculture practices</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>8 Symbiobacterium terraclitae</t>
+          <t>Symbiobacterium terraclitae</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Thermophilic bacterium that degrades organic matter and participates in symbiotic relationships with other microorganisms</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bioremediation of contaminated soil, production of bioactive compounds, and development of novel biofertilizers</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>9 Ilumatobacter fluminis</t>
+          <t>Ilumatobacter fluminis</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Ilumatobacter fluminis is a bacterium that plays a role in the degradation of organic matter and production of bioactive compounds</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>It can be used for bioremediation, production of biofertilizers, and development of eco-friendly agricultural practices</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>10 Filomicrobium insigne</t>
+          <t>Filomicrobium insigne</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Filomicrobium insigne is a bacterium that plays a role in the degradation of organic matter and has been found in various environments, including soil and water. It is a microaerophile, requiring low oxygen levels to grow, and is capable of fixing nitrogen, solubilizing phosphorus, and producing plant growth-promoting substances.</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Filomicrobium insigne can be used for sustainable bioprospecting in agriculture, particularly in the development of biofertilizers and biostimulants. Its ability to fix nitrogen and solubilize phosphorus makes it a potential candidate for reducing the use of synthetic fertilizers, while its production of plant growth-promoting substances can enhance crop yields and plant health. Additionally, its microaerophilic nature makes it suitable for use in low-oxygen environments, such as in soil or aquatic ecosystems.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>11 Fischerella indica</t>
+          <t>Fischerella indica</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Nitrogen fixation, production of bioactive compounds, and plant growth promotion</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Biofertilizer development, bioremediation, and production of eco-friendly agricultural chemicals</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>12 Anaerolinea thermophila</t>
+          <t>Anaerolinea thermophila</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Anaerolinea thermophila is a thermophilic, anaerobic bacterium that plays a key role in the degradation of organic matter and production of bioactive compounds</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>It can be used for sustainable bioprospecting in the production of biofuels, bioplastics, and other eco-friendly technologies, as well as in the development of novel agricultural practices such as bioremediation and biofertilization</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>13 Rhodoplanes tepidicaeni</t>
+          <t>Rhodoplanes tepidicaeni</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Phototrophic bacterium capable of producing pigments and fixing nitrogen</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Potential applications in bioremediation, biofertilizers, and production of natural pigments for eco-friendly industries</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>14 Gaiella occulta</t>
+          <t>Gaiella occulta</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Gaiella occulta is an actinobacterium with potential applications in biodegradation and production of bioactive compounds</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>It can be used for eco-friendly tech such as bioremediation of pollutants and production of natural products, as well as in agriculture for plant growth promotion and biocontrol</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>15 Mycolicibacterium confluentis</t>
+          <t>Mycolicibacterium confluentis</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Mycolicibacterium confluentis is a species of bacteria that plays a role in the degradation of organic matter and has been found in various environments, including soil and water. It is also known to have potential applications in bioremediation and the production of bioactive compounds.</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Mycolicibacterium confluentis can be used for sustainable bioprospecting in the development of eco-friendly technologies, such as biodegradation of pollutants, production of biofertilizers, and the creation of novel bioactive compounds for agricultural and pharmaceutical applications.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>16 Hyphomicrobium chloromethanicum</t>
+          <t>Hyphomicrobium chloromethanicum</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Methane oxidation and methylotrophy, contributing to the global carbon cycle</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bioremediation of contaminated environments, production of single-cell protein for animal feed, and development of biofilters for air pollution control</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>17 Psychroglaciecola arctica</t>
+          <t>Psychroglaciecola arctica</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Psychrotrophic bacterium with potential for biodegradation and production of cold-active enzymes</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bioremediation of cold environments, production of bioactive compounds, and development of sustainable agricultural practices in cold climates</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>18 Ornithinimicrobium laminariae</t>
+          <t>Ornithinimicrobium laminariae</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Decomposition and nutrient cycling in marine ecosystems</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bioremediation of pollutants, production of bioactive compounds, and potential use in seaweed-based agriculture</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>19 Pedomicrobium manganicum</t>
+          <t>Pedomicrobium manganicum</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Manganese oxidation, contributing to the formation of manganese oxides and influencing metal cycling in the environment</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bioremediation of heavy metals, improvement of soil quality, and potential application in the development of eco-friendly technologies for metal recovery and wastewater treatment</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>20 Desulfomonile limimaris</t>
+          <t>Desulfomonile limimaris</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Sulfur-reducing bacterium, contributes to sulfur cycle in marine environments</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bioremediation of sulfur-polluted sites, potential for biofuel production and soil amendment in agriculture</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>21 Iamia majanohamensis</t>
+          <t>Iamia majanohamensis</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Marine bacterium with potential for biodegradation and production of bioactive compounds</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bioremediation of marine pollutants, production of natural products for agriculture and pharmaceuticals</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>22 Ktedonosporobacter rubrisoli</t>
+          <t>Ktedonosporobacter rubrisoli</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Soil bacterium with potential for plant growth promotion and nitrogen fixation</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Biofertilizer development, soil remediation, and sustainable agriculture practices</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>23 Hydrogenispora ethanolica</t>
+          <t>Hydrogenispora ethanolica</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Thermophilic, hydrogen-producing bacterium that plays a role in the degradation of organic matter and production of biofuels</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Production of biohydrogen, bioremediation of pollutants, and development of sustainable biofuel technologies</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>24 Hoeflea prorocentri</t>
+          <t>Hoeflea prorocentri</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Nitrogen fixation, symbiotic relationships with dinoflagellates, and potential production of bioactive compounds</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Biofertilizers, bioremediation, and development of novel antimicrobial agents or pigments for eco-friendly industries</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>25 Rhabdothermincola salaria</t>
+          <t>Rhabdothermincola salaria</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Rhabdothermincola salaria is a thermophilic bacterium that plays a role in the degradation of organic matter and production of bioactive compounds</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>It can be used for the development of eco-friendly technologies such as bioremediation, biofuel production, and sustainable agriculture practices</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>26 Romboutsia hominis</t>
+          <t>Romboutsia hominis</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Romboutsia hominis is a butyrate-producing bacterial species, primarily found in the human gut microbiome, contributing to gut health and potentially influencing host metabolism and immune system</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Romboutsia hominis can be utilized for sustainable bioprospecting in the development of eco-friendly probiotics, animal feed additives, and biofertilizers, promoting a balanced gut microbiome and reducing the need for synthetic additives in agriculture</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>27 Aquihabitans daechungensis</t>
+          <t>Aquihabitans daechungensis</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Degradation of organic pollutants and production of bioactive compounds</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bioremediation of contaminated environments, production of natural antimicrobials and antifungals for agricultural use</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>28 Nostocoides japonicum</t>
+          <t>Nostocoides japonicum</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Nitrogen fixation, decomposition, and production of extracellular polymeric substances</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Wastewater treatment, bioremediation, and biofertilizer production for sustainable agriculture</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>29 Flexilinea flocculi</t>
+          <t>Flexilinea flocculi</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Flexilinea flocculi is a type of bacterium that plays a role in the decomposition of organic matter and has been found in various environments, including soil and freshwater sediments. It is capable of producing bioactive compounds and has potential applications in biotechnology and environmental remediation.</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Flexilinea flocculi can be used for sustainable bioprospecting, such as the production of biofertilizers, biodegradation of pollutants, and the development of novel antimicrobial compounds. Its ability to thrive in diverse environments makes it a promising candidate for eco-friendly technologies and agricultural applications.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>30 Corynebacterium xerosis</t>
+          <t>Corynebacterium xerosis</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Corynebacterium xerosis is a Gram-positive, rod-shaped bacterium that plays a role in the decomposition of organic matter and has been found in various environments, including soil, water, and as part of the human microbiome. It has also been implicated in the production of bioactive compounds and has potential applications in biotechnology.</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Corynebacterium xerosis can be used for sustainable bioprospecting in the production of biofertilizers, biodegradation of pollutants, and the development of novel bioactive compounds for agricultural and pharmaceutical applications, contributing to eco-friendly technologies and sustainable agriculture practices.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>31 Candidatus Thiodictyon syntrophicum</t>
+          <t>Candidatus Thiodictyon syntrophicum</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Sulfur-reducing bacterium that plays a key role in the sulfur cycle, contributing to the degradation of organic matter and the release of sulfur compounds</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Potential applications in bioremediation of sulfur-polluted environments, production of biofuels, and improvement of agricultural soil health through sulfur cycling</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1123,259 +1123,259 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>32 Corynebacterium incognita</t>
+          <t>Corynebacterium incognita</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Corynebacterium incognita is a Gram-positive, rod-shaped bacterium that has been isolated from various environments, including soil and plant tissues. Its primary function is to decompose organic matter and fix nitrogen, contributing to nutrient cycling in ecosystems.</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Corynebacterium incognita can be used for sustainable bioprospecting in agriculture, particularly in the development of biofertilizers and biostimulants that promote plant growth and reduce the need for synthetic fertilizers.</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>33 Andreesenia angusta</t>
+          <t>Andreesenia angusta</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Andreesenia angusta is a psychrotolerant bacterium that plays a role in decomposing organic matter and fixing nitrogen in cold environments</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>It can be used for eco-friendly tech such as bioremediation of cold polluted sites, and in agriculture for improving soil fertility and plant growth in low-temperature conditions</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>34 Nigerium massiliense</t>
+          <t>Nigerium massiliense</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Nigerium massiliense is a bacterium that has been found to have potential applications in bioremediation and the production of bioactive compounds, with a role in decomposing organic matter and fixing nitrogen</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>It can be used for eco-friendly technologies such as biodegradation of pollutants, production of biofertilizers, and development of novel antimicrobial agents, contributing to sustainable agriculture and environmental remediation</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>35 Conexibacter arvalis</t>
+          <t>Conexibacter arvalis</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Soil bacterium with potential for biodegradation and plant growth promotion</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bioremediation of pollutants, production of biofertilizers, and development of sustainable agricultural practices</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>36 Miltoncostaea oceani</t>
+          <t>Miltoncostaea oceani</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Miltoncostaea oceani is a marine bacterium that plays a role in the degradation of organic matter and production of bioactive compounds</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>It can be used for the development of eco-friendly technologies such as bioremediation of pollutants, production of biofertilizers, and discovery of novel antimicrobial compounds</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>37 Rhabdothermincola sediminis</t>
+          <t>Rhabdothermincola sediminis</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Rhabdothermincola sediminis is a thermophilic bacterium that plays a role in the degradation of organic matter and production of bioactive compounds</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>It can be used for bioremediation of polluted environments, production of biofuels, and development of novel therapeutics and agricultural products</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>38 Pseudolabrys taiwanensis</t>
+          <t>Pseudolabrys taiwanensis</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Pseudolabrys taiwanensis is a rhizobial bacterium that plays a crucial role in nitrogen fixation, solubilizing phosphorus, and producing plant growth-promoting substances, which can enhance plant growth and soil fertility</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>It can be used as a biofertilizer to reduce the use of chemical fertilizers, promote sustainable agriculture, and improve soil health, thereby contributing to eco-friendly agricultural practices</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>39 Dichotomicrobium thermohalophilum</t>
+          <t>Dichotomicrobium thermohalophilum</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Nitrogen fixation, organic matter decomposition, and participation in microbial communities in saline environments</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bioremediation of polluted saline soils, production of biofertilizers, and development of novel enzymes for industrial applications</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>40 Streptomyces antibioticus</t>
+          <t>Streptomyces antibioticus</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Production of antibiotics and secondary metabolites with antimicrobial and antifungal properties</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Biodegradation of pollutants, plant growth promotion, and biocontrol of plant pathogens for eco-friendly agriculture</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>41 Roseitalea porphyridii</t>
+          <t>Roseitalea porphyridii</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Phototrophic bacterium involved in the degradation of organic matter and production of pigments</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Potential applications in bioremediation, biofertilizers, and production of natural pigments for the food and cosmetic industries</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>42 Lignipirellula cremea</t>
+          <t>Lignipirellula cremea</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Lignipirellula cremea is a bacterium that plays a role in the degradation of lignin, a complex organic polymer found in plant cell walls, contributing to the carbon cycle and potentially to the production of biofuels and other bioproducts</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>It can be used for eco-friendly technologies such as biofuel production, bioremediation of polluted environments, and development of sustainable agricultural practices through the enhancement of plant biomass degradation and nutrient cycling</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>43 Zhenhengia yiwuensis</t>
+          <t>Zhenhengia yiwuensis</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Decomposition and nutrient cycling in soil ecosystems</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bioremediation, organic fertilizer production, and soil health improvement for sustainable agriculture</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1387,853 +1387,853 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>44 Microbaculum marinum</t>
+          <t>Microbaculum marinum</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Microbaculum marinum is a Gram-negative, aerobic, rod-shaped bacterium that has been found to degrade polycyclic aromatic hydrocarbons (PAHs) and other organic pollutants, suggesting a role in bioremediation and environmental cleanup</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>This species can be utilized for the development of sustainable bioremediation technologies, such as cleaning up contaminated soil and water, and also has potential applications in the production of biofuels and bioproducts</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>45 Sporobacter termitidis</t>
+          <t>Sporobacter termitidis</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Cellulose degradation and fermentation in the hindgut of termites</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Production of biofuels, biogas, and other value-added chemicals from lignocellulosic biomass</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>46 Parasynechococcus marenigrum</t>
+          <t>Parasynechococcus marenigrum</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Photosynthetic cyanobacterium contributing to global carbon cycling and primary production in marine ecosystems</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Potential applications in biofertilizers, bioremediation of pollutants, and production of bioactive compounds for pharmaceutical or agricultural uses</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>47 Simkania negevensis</t>
+          <t>Simkania negevensis</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Chlamydia-like obligate intracellular bacterium, potentially involved in respiratory infections and possibly influencing microbial communities</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bioremediation, biofertilization, or biopesticide development due to its unique metabolic capabilities and potential to interact with various microbial consortia</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-2</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>48 Hyphomicrobium sulfonivorans</t>
+          <t>Hyphomicrobium sulfonivorans</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Hyphomicrobium sulfonivorans is a Gram-negative, aerobic, and methylotrophic bacterium that plays a key role in the degradation of organic sulfur compounds, contributing to the global sulfur cycle and potentially remediating polluted environments</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>This species can be utilized for bioremediation of sulfur-polluted sites, production of biofertilizers, and development of sustainable technologies for the removal of sulfur-containing pollutants from wastewater and soil, promoting eco-friendly agriculture and environmental conservation</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>49 Prochlorococcus marinus</t>
+          <t>Prochlorococcus marinus</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Photosynthetic cyanobacterium, primary producer in ocean ecosystems, contributes to global carbon cycle and oxygen production</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Potential applications in eco-friendly tech include biofuel production, carbon sequestration, and nutrient cycling for sustainable agriculture</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>50 Hyphomicrobium album</t>
+          <t>Hyphomicrobium album</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Methane oxidation, nitrogen fixation, and degradation of organic pollutants</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bioremediation of contaminated soil and water, production of biofertilizers, and development of sustainable methane-based bioenergy systems</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>51 Mycobacterium conspicuum</t>
+          <t>Mycobacterium conspicuum</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Mycobacterium conspicuum is a non-tuberculous mycobacterium that has been isolated from various environmental sources, including soil and water, and has been found to have potential applications in bioremediation and biodegradation of pollutants</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>It can be used for the biodegradation of polycyclic aromatic hydrocarbons (PAHs) and other organic pollutants, making it a potential tool for eco-friendly bioremediation technologies and sustainable agriculture practices</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-2</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>52 Salaquimonas pukyongi</t>
+          <t>Salaquimonas pukyongi</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Polycyclic aromatic hydrocarbon degradation and potential role in marine ecosystem balance</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bioremediation of polluted marine environments, enhancement of oil spill cleanup, and possible applications in eco-friendly agricultural practices</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>53 Clostridium estertheticum</t>
+          <t>Clostridium estertheticum</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Psychrotolerant, anaerobic, spore-forming bacterium involved in spoilage of chilled meats and capable of producing ester compounds</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Potential applications in biodegradation, biofuel production, and development of novel enzymes for eco-friendly industrial processes</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-2</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>54 Pelolinea submarina</t>
+          <t>Pelolinea submarina</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Pelolinea submarina is a bacterium that plays a role in the sulfur cycle, contributing to the degradation of organic matter and the production of sulfide</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>It can be used for bioremediation of polluted environments, such as sediment and water, and has potential applications in sustainable agriculture and eco-friendly technologies, such as biofertilizers and biostimulants</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>55 Afifella pfennigii</t>
+          <t>Afifella pfennigii</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Nitrogen fixation, carbon sequestration, and production of bioactive compounds</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Biofertilizers, bioremediation, and production of sustainable biofuels and chemicals</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>56 Bauldia consociata</t>
+          <t>Bauldia consociata</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Nitrogen fixation, plant growth promotion, and biocontrol of plant pathogens</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Biofertilizer production, phytoremediation, and development of eco-friendly pesticides</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>57 Hyphomicrobium hollandicum</t>
+          <t>Hyphomicrobium hollandicum</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Methane oxidation, nitrogen fixation, and degradation of organic pollutants</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bioremediation of contaminated soil and water, production of biofertilizers, and development of methane-based biofuels</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>58 Miltoncostaea marina</t>
+          <t>Miltoncostaea marina</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Miltoncostaea marina is a marine bacterium that plays a role in the degradation of organic matter and production of bioactive compounds</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>It can be used for the development of eco-friendly technologies such as bioremediation of pollutants, production of biofertilizers, and discovery of novel antimicrobial compounds</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>59 Mycetocola tolaasinivorans</t>
+          <t>Mycetocola tolaasinivorans</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Mycetocola tolaasinivorans is a bacterium that degrades tolaasin, a toxin produced by the fungus Pseudomonas tolaasii, which causes brown blotch disease in mushrooms. It plays a role in the degradation of toxic compounds and has potential applications in bioremediation.</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Mycetocola tolaasinivorans can be used for sustainable bioprospecting in the development of eco-friendly technologies for the degradation of toxic pollutants, and in agriculture for the control of plant diseases caused by Pseudomonas species.</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>60 Waddlia chondrophila</t>
+          <t>Waddlia chondrophila</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Intracellular bacterial pathogen, potential role in reproductive tract infections and abortion in cattle</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Biodegradation and bioremediation of environmental pollutants, potential use in veterinary medicine for development of vaccines or diagnostic tools</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-2</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>61 Algorimarina butyrica</t>
+          <t>Algorimarina butyrica</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Fermentation and production of butyric acid, a compound with potential applications in food, pharmaceutical, and biofuel industries</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Production of biodegradable plastics, animal feed, and biofuels, as well as potential use in agriculture as a biofertilizer or soil conditioner</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>62 Bellilinea caldifistulae</t>
+          <t>Bellilinea caldifistulae</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Thermophilic, anaerobic, and cellulolytic bacterium that degrades cellulose and produces biofuels and other valuable compounds</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Production of biofuels, bioproducts, and biofertilizers, as well as bioremediation of polluted environments and improvement of soil health</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>63 Caldilinea tarbellica</t>
+          <t>Caldilinea tarbellica</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Fermentation and organic matter decomposition in aquatic environments</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bioremediation of polluted water, production of biofuels and bioproducts, and enhancement of soil fertility</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>64 Bauldia litoralis</t>
+          <t>Bauldia litoralis</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Nitrogen fixation, organic matter decomposition, and production of antimicrobial compounds</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Biofertilizers, bioremediation of polluted soils, and development of novel antimicrobial agents for eco-friendly agriculture and medicine</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>65 Phycicoccus endophyticus</t>
+          <t>Phycicoccus endophyticus</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Plant growth promotion, biocontrol, and production of secondary metabolites</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Biofertilizer, bioremediation, and production of eco-friendly chemicals</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>66 Desulfatitalea tepidiphila</t>
+          <t>Desulfatitalea tepidiphila</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Sulfur-reducing bacterium, involved in the degradation of organic matter and sulfur compounds in anoxic environments</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bioremediation of contaminated soil and groundwater, production of biofuels, and potential use in microbial fuel cells for sustainable energy generation</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>67 Thermogutta terrifontis</t>
+          <t>Thermogutta terrifontis</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Thermogutta terrifontis is a thermophilic bacterium that plays a role in decomposing organic matter and fixing nitrogen in high-temperature environments</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>It can be used for bioremediation of polluted soil and water, production of biofertilizers, and development of novel thermostable enzymes for eco-friendly industrial processes</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>68 Pseudorhodoplanes sinuspersici</t>
+          <t>Pseudorhodoplanes sinuspersici</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Nitrogen fixation, production of plant growth-promoting substances, and potential for biodegradation of pollutants</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Biofertilizers, bioremediation of contaminated soil and water, and development of sustainable agricultural practices</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>69 Oceanirhabdus sediminicola</t>
+          <t>Oceanirhabdus sediminicola</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Marine bacterium with potential for biodegradation and production of bioactive compounds</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bioremediation of polluted marine environments, production of natural products for agriculture and pharmaceuticals</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>70 Thiorhodococcus minor</t>
+          <t>Thiorhodococcus minor</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Sulfur-oxidizing bacterium, plays a role in the sulfur cycle and can be used for bioremediation of sulfur-containing pollutants</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Potential application in eco-friendly technologies such as bioremediation of polluted environments, bioleaching of metals, and production of biofertilizers</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>71 Desulfomonile tiedjei</t>
+          <t>Desulfomonile tiedjei</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Reductive dehalogenation of chlorinated compounds</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bioremediation of contaminated soil and groundwater, potential for use in eco-friendly degradation of pollutants</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-2</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>72 Waddlia malaysiensis</t>
+          <t>Waddlia malaysiensis</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Chlamydia-like obligate intracellular bacterium, potentially involved in amoebal endosymbiosis and influencing microbial community dynamics</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bioremediation of wastewater, biocontrol of plant pathogens, and development of novel antimicrobial compounds</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-2</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>73 Konateibacter massiliensis</t>
+          <t>Konateibacter massiliensis</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Konateibacter massiliensis is a Gram-negative, aerobic, rod-shaped bacterium with potential applications in biodegradation and bioremediation of pollutants</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>It can be used for the development of eco-friendly technologies for the cleanup of contaminated environments, such as soil and water, and may also have applications in sustainable agriculture practices</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>74 Pirellulimonas nuda</t>
+          <t>Pirellulimonas nuda</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Pirellulimonas nuda is a species of bacteria that has been found to have a role in the degradation of organic pollutants and production of bioactive compounds</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>It can be used for bioremediation of contaminated soil and water, and for the production of eco-friendly agricultural products such as biofertilizers and biopesticides</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>75 Rhodoplanes pokkaliisoli</t>
+          <t>Rhodoplanes pokkaliisoli</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Nitrogen fixation, photosynthesis, and production of pigments and bioactive compounds</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Biofertilizer production, biodegradation of pollutants, and development of natural food colorants and pharmaceuticals</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>76 Rosistilla oblonga</t>
+          <t>Rosistilla oblonga</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Marine bacterium contributing to the degradation of organic matter and production of bioactive compounds</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Potential applications in bioremediation, biofertilizers, and production of natural products for pharmaceutical or agricultural use</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>77 Woeseia oceani</t>
+          <t>Woeseia oceani</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Nitrogen fixation, carbon cycling, and production of bioactive compounds</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Marine biotechnology, biofertilizers, and bioremediation of polluted environments</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>78 Vampirovibrio chlorellavorus</t>
+          <t>Vampirovibrio chlorellavorus</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Parasitic bacterium that infects and lyses Chlorella algae cells, potentially useful for biocontrol of algal blooms</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bioremediation of algal blooms, production of biofuels, and development of sustainable algal-based agricultural systems</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>79 Clostridium perfringens</t>
+          <t>Clostridium perfringens</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Clostridium perfringens is a Gram-positive, anaerobic, spore-forming bacterium that plays a significant role in decomposing organic matter and producing toxins that can cause food poisoning and gas gangrene in humans</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>It can be used for biogas production, as a probiotic in animal feed, and for the development of eco-friendly pesticides and fertilizers</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-2</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>80 Staphylococcus gallinarum</t>
+          <t>Staphylococcus gallinarum</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Staphylococcus gallinarum is a coagulase-negative bacterium commonly found on the skin and mucous membranes of chickens, playing a role in the microbiome and potentially contributing to disease resistance</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>It can be used for the development of probiotics, antimicrobial peptides, and other eco-friendly technologies to improve poultry health and reduce the need for antibiotics in agriculture</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>81 Raineyella fluvialis</t>
+          <t>Raineyella fluvialis</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Raineyella fluvialis is a Gram-positive, rod-shaped bacterium involved in the degradation of organic pollutants and production of bioactive compounds</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>It can be used for bioremediation of contaminated environments, production of biofertilizers, and development of sustainable agricultural practices</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>82 Symmachiella dynata</t>
+          <t>Symmachiella dynata</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Cyanobacterium with potential for nitrogen fixation and production of bioactive compounds</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Biofertilizer development, bioremediation, and production of natural products for agriculture and pharmaceutical industries</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2245,325 +2245,325 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>83 Aliiruegeria lutimaris</t>
+          <t>Aliiruegeria lutimaris</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Aliiruegeria lutimaris is a Gram-negative, aerobic, and rod-shaped bacterium that has been found to have potential applications in bioremediation and biodegradation of pollutants</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>It can be used for the biodegradation of organic pollutants, such as polycyclic aromatic hydrocarbons (PAHs) and heavy metals, making it a potential tool for eco-friendly cleanup of contaminated sites and sustainable agriculture practices</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>84 Thermanaerothrix daxensis</t>
+          <t>Thermanaerothrix daxensis</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Thermanaerothrix daxensis is a thermophilic bacterium that plays a role in the degradation of organic matter and production of bioactive compounds</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>It can be used for bioremediation of polluted environments, production of biofuels, and development of novel thermostable enzymes for eco-friendly industrial applications</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>85 Actinoplanes siamensis</t>
+          <t>Actinoplanes siamensis</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Soil-dwelling bacterium with potential for biodegradation and production of secondary metabolites</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Can be used for eco-friendly bioremediation of pollutants, production of bioactive compounds, and development of sustainable agricultural practices</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>86 Thiohalocapsa halophila</t>
+          <t>Thiohalocapsa halophila</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Sulfur-oxidizing bacterium that plays a key role in the sulfur cycle, contributing to the degradation of organic matter and the formation of sulfur compounds</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Has potential applications in bioremediation of polluted environments, bioleaching of metals, and production of biofertilizers and biopesticides for sustainable agriculture</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>87 Symbioplanes lichenis</t>
+          <t>Symbioplanes lichenis</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Symbioplanes lichenis is a bacterium that has been found to have a symbiotic relationship with lichens, contributing to nutrient cycling and potentially producing secondary metabolites with antimicrobial properties</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>This species can be utilized for the development of sustainable agricultural practices, such as biofertilizers or biopesticides, and may also have applications in the production of eco-friendly compounds for the pharmaceutical or chemical industries</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>88 Aureliella helgolandensis</t>
+          <t>Aureliella helgolandensis</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Marine alphaproteobacterium with potential for biodegradation and production of bioactive compounds</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bioremediation of marine pollutants, production of antimicrobial compounds, and development of sustainable aquaculture practices</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>89 Hansschlegelia zhihuaiae</t>
+          <t>Hansschlegelia zhihuaiae</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Denitrification and nitrogen cycling</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bioremediation of nitrate-polluted water and soil, sustainable agriculture through biofertilizers</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>90 Romboutsia lituseburensis</t>
+          <t>Romboutsia lituseburensis</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Romboutsia lituseburensis is a spore-forming bacterium that plays a role in the degradation of organic matter and production of antimicrobial compounds</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>It can be used for the development of eco-friendly bioproducts, such as biofertilizers, biopesticides, and bioremediation agents, due to its ability to produce antimicrobial compounds and degrade organic pollutants</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>91 Posidoniimonas corsicana</t>
+          <t>Posidoniimonas corsicana</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Posidoniimonas corsicana is a bacterium that has been found to play a role in the degradation of organic matter and production of bioactive compounds, with potential applications in bioremediation, agriculture, and pharmaceutical industries</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>It can be used for eco-friendly technologies such as biodegradation of pollutants, production of biofertilizers, and development of sustainable agricultural practices</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>92 Clostridium chrysemydis</t>
+          <t>Clostridium chrysemydis</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Clostridium chrysemydis is a bacterium that plays a role in the decomposition of organic matter and production of bioactive compounds</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>It can be used for bioremediation, production of biofuels, and development of eco-friendly agricultural products</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>93 Microbacterium halophilum</t>
+          <t>Microbacterium halophilum</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Microbacterium halophilum is a Gram-positive, rod-shaped bacterium that plays a role in the degradation of organic matter and production of extracellular enzymes, and has potential applications in bioremediation and biofertilization</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>It can be used for eco-friendly technologies such as biodegradation of pollutants, production of bioactive compounds, and development of sustainable agricultural practices, including plant growth promotion and soil remediation</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>94 Thiococcus pfennigii</t>
+          <t>Thiococcus pfennigii</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Sulfur-reducing bacterium, plays a role in the sulfur cycle, and contributes to the degradation of organic matter</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Potential applications in bioremediation of polluted environments, production of biofuels, and sustainable agriculture through improved soil fertility and plant growth promotion</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>95 Solirubrobacter soli</t>
+          <t>Solirubrobacter soli</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Solirubrobacter soli is a Gram-positive, aerobic bacterium that plays a role in soil ecosystem functioning, particularly in the decomposition of organic matter and the cycling of nutrients</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>It has potential applications in sustainable agriculture, such as plant growth promotion, biofertilization, and bioremediation of contaminated soils, as well as in the development of eco-friendly technologies for waste management and environmental remediation</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>96 Mycolicibacterium gadium</t>
+          <t>Mycolicibacterium gadium</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Mycolicibacterium gadium is a species of bacteria that plays a role in the degradation of organic matter and has been found in various environments, including soil and water. It is also known to have potential applications in bioremediation and the production of bioactive compounds.</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Mycolicibacterium gadium can be used for sustainable bioprospecting in the development of eco-friendly technologies, such as biodegradation of pollutants, production of biofertilizers, and creation of novel bioactive compounds for agricultural and pharmaceutical applications.</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>97 Oricola indica</t>
+          <t>Oricola indica</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Oricola indica is a bacterium that has been found to have potential applications in bioremediation, plant growth promotion, and production of bioactive compounds</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>It can be used for eco-friendly technologies such as biodegradation of pollutants, production of biofertilizers, and development of sustainable agricultural practices</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -2575,66 +2575,66 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>98 Clostridium paraputrificum</t>
+          <t>Clostridium paraputrificum</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Clostridium paraputrificum is a Gram-positive, anaerobic bacterium that plays a significant role in the decomposition of organic matter and production of short-chain fatty acids, particularly butyric acid, through fermentation processes.</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>This species has potential applications in sustainable bioprospecting, including the production of biofuels, biodegradation of pollutants, and improvement of soil health through the production of plant growth-promoting substances.</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-2</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>99 Candidatus Protochlamydia naegleriophila</t>
+          <t>Candidatus Protochlamydia naegleriophila</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Endosymbiont of the amoeba Naegleria, potentially influencing its host's ecology and contributing to nutrient cycling in aquatic environments</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bioremediation, biofertilization, and wastewater treatment due to its potential to degrade organic pollutants and promote nutrient cycling</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>100 Jatrophihabitans telluris</t>
+          <t>Jatrophihabitans telluris</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Error / Extraction Failed</t>
+          <t>Plant growth promotion, nitrogen fixation, and production of antimicrobial compounds</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Biofertilizer development, phytoremediation, and biological control of plant pathogens for eco-friendly agriculture</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BSL-1</t>
         </is>
       </c>
     </row>

</xml_diff>